<commit_message>
Phat hien moi ve init baudrate
</commit_message>
<xml_diff>
--- a/SHT-RS485-Modbus-RTU-Temperature-Humidity-Sensor/SHT40-IP67-RS485_RS485-TTL_USB-TTL.xlsx
+++ b/SHT-RS485-Modbus-RTU-Temperature-Humidity-Sensor/SHT40-IP67-RS485_RS485-TTL_USB-TTL.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Git\Github\longhoney\KhaoSat_RS485-Modbus\SHT-RS485-Modbus-RTU-Temperature-Humidity-Sensor\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Git\Github\longhoney\KhaoSat_RS485-Modbus_1\SHT-RS485-Modbus-RTU-Temperature-Humidity-Sensor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4737AFE5-AD38-4B76-BB58-4D81EA883B52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF7C3BF5-BF22-4C96-8B65-B4003F57537F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Read_Data" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="92">
   <si>
     <t>Address code</t>
   </si>
@@ -216,9 +216,6 @@
     <t>Value of Baudrate</t>
   </si>
   <si>
-    <t>{01}{03}{02}{00}{01}{79}{84}</t>
-  </si>
-  <si>
     <t>Địa chỉ: 1- 254</t>
   </si>
   <si>
@@ -301,6 +298,12 @@
   </si>
   <si>
     <t>(Chỉ 3 cái nên có thể dò với lệnh đọc địa chỉ là đủ)</t>
+  </si>
+  <si>
+    <t>{07}{03}{02}{00}{07}{71}{86}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.binaryhexconverter.com/decimal-to-hex-converter </t>
   </si>
 </sst>
 </file>
@@ -532,7 +535,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -552,6 +555,23 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -570,18 +590,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -589,15 +597,8 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -898,7 +899,7 @@
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="17" t="s">
         <v>8</v>
       </c>
       <c r="B3" t="s">
@@ -930,34 +931,34 @@
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A4" s="22"/>
-      <c r="C4" s="13" t="s">
+      <c r="A4" s="17"/>
+      <c r="C4" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="F4" s="16"/>
-      <c r="G4" s="15" t="s">
+      <c r="F4" s="23"/>
+      <c r="G4" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="H4" s="16"/>
-      <c r="I4" s="19" t="s">
+      <c r="H4" s="23"/>
+      <c r="I4" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="J4" s="20"/>
+      <c r="J4" s="19"/>
     </row>
     <row r="5" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="22"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="18"/>
+      <c r="A5" s="17"/>
+      <c r="C5" s="21"/>
+      <c r="D5" s="21"/>
+      <c r="E5" s="24"/>
+      <c r="F5" s="25"/>
+      <c r="G5" s="24"/>
+      <c r="H5" s="25"/>
       <c r="I5" s="6" t="s">
         <v>36</v>
       </c>
@@ -966,7 +967,7 @@
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A6" s="22"/>
+      <c r="A6" s="17"/>
       <c r="C6" s="8" t="s">
         <v>54</v>
       </c>
@@ -986,10 +987,10 @@
         <v>6</v>
       </c>
       <c r="I6" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="J6" s="8" t="s">
         <v>66</v>
-      </c>
-      <c r="J6" s="8" t="s">
-        <v>67</v>
       </c>
       <c r="M6" t="s">
         <v>11</v>
@@ -1002,10 +1003,10 @@
       <c r="G7" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I7" s="25" t="s">
-        <v>65</v>
-      </c>
-      <c r="J7" s="25"/>
+      <c r="I7" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="J7" s="16"/>
       <c r="M7" t="s">
         <v>39</v>
       </c>
@@ -1022,10 +1023,10 @@
         <v>10</v>
       </c>
       <c r="H8" t="s">
+        <v>86</v>
+      </c>
+      <c r="K8" t="s">
         <v>87</v>
-      </c>
-      <c r="K8" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.35">
@@ -1053,7 +1054,7 @@
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.35">
@@ -1090,36 +1091,36 @@
       <c r="A14" t="s">
         <v>19</v>
       </c>
-      <c r="C14" s="21" t="s">
+      <c r="C14" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="D14" s="21" t="s">
+      <c r="D14" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="E14" s="21" t="s">
+      <c r="E14" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="F14" s="21" t="s">
+      <c r="F14" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="G14" s="21"/>
-      <c r="H14" s="21" t="s">
+      <c r="G14" s="15"/>
+      <c r="H14" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="I14" s="21"/>
-      <c r="J14" s="21" t="s">
+      <c r="I14" s="15"/>
+      <c r="J14" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="K14" s="21"/>
+      <c r="K14" s="15"/>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="C15" s="21"/>
-      <c r="D15" s="21"/>
-      <c r="E15" s="21"/>
-      <c r="F15" s="21"/>
-      <c r="G15" s="21"/>
-      <c r="H15" s="21"/>
-      <c r="I15" s="21"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="15"/>
+      <c r="H15" s="15"/>
+      <c r="I15" s="15"/>
       <c r="J15" s="6" t="s">
         <v>36</v>
       </c>
@@ -1173,7 +1174,7 @@
       </c>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A21" s="22" t="s">
+      <c r="A21" s="17" t="s">
         <v>8</v>
       </c>
       <c r="B21" t="s">
@@ -1205,34 +1206,34 @@
       </c>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A22" s="22"/>
-      <c r="C22" s="13" t="s">
+      <c r="A22" s="17"/>
+      <c r="C22" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="D22" s="13" t="s">
+      <c r="D22" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="E22" s="15" t="s">
+      <c r="E22" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="F22" s="16"/>
-      <c r="G22" s="15" t="s">
+      <c r="F22" s="23"/>
+      <c r="G22" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="H22" s="16"/>
-      <c r="I22" s="19" t="s">
+      <c r="H22" s="23"/>
+      <c r="I22" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="J22" s="20"/>
+      <c r="J22" s="19"/>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A23" s="22"/>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="17"/>
-      <c r="F23" s="18"/>
-      <c r="G23" s="17"/>
-      <c r="H23" s="18"/>
+      <c r="A23" s="17"/>
+      <c r="C23" s="21"/>
+      <c r="D23" s="21"/>
+      <c r="E23" s="24"/>
+      <c r="F23" s="25"/>
+      <c r="G23" s="24"/>
+      <c r="H23" s="25"/>
       <c r="I23" s="6" t="s">
         <v>36</v>
       </c>
@@ -1241,7 +1242,7 @@
       </c>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A24" s="22"/>
+      <c r="A24" s="17"/>
       <c r="C24" s="8" t="s">
         <v>54</v>
       </c>
@@ -1261,18 +1262,18 @@
         <v>2</v>
       </c>
       <c r="I24" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="J24" s="8" t="s">
         <v>70</v>
-      </c>
-      <c r="J24" s="8" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="25" spans="1:16" ht="14.5" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B25" s="3"/>
-      <c r="I25" s="25" t="s">
-        <v>69</v>
-      </c>
-      <c r="J25" s="25"/>
+      <c r="I25" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="J25" s="16"/>
     </row>
     <row r="26" spans="1:16" ht="29" x14ac:dyDescent="0.35">
       <c r="A26" s="7" t="s">
@@ -1286,7 +1287,7 @@
         <v>10</v>
       </c>
       <c r="H26" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="27" spans="1:16" ht="14.5" customHeight="1" x14ac:dyDescent="0.5">
@@ -1317,7 +1318,7 @@
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.35">
@@ -1350,30 +1351,30 @@
       <c r="A32" t="s">
         <v>19</v>
       </c>
-      <c r="C32" s="21" t="s">
+      <c r="C32" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="D32" s="21" t="s">
+      <c r="D32" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="E32" s="21" t="s">
+      <c r="E32" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="F32" s="23" t="s">
+      <c r="F32" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="G32" s="24"/>
-      <c r="H32" s="19" t="s">
+      <c r="G32" s="27"/>
+      <c r="H32" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="I32" s="20"/>
+      <c r="I32" s="19"/>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="C33" s="21"/>
-      <c r="D33" s="21"/>
-      <c r="E33" s="21"/>
-      <c r="F33" s="23"/>
-      <c r="G33" s="24"/>
+      <c r="C33" s="15"/>
+      <c r="D33" s="15"/>
+      <c r="E33" s="15"/>
+      <c r="F33" s="26"/>
+      <c r="G33" s="27"/>
       <c r="H33" s="6" t="s">
         <v>36</v>
       </c>
@@ -1422,7 +1423,7 @@
       </c>
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A39" s="22" t="s">
+      <c r="A39" s="17" t="s">
         <v>8</v>
       </c>
       <c r="B39" t="s">
@@ -1454,34 +1455,34 @@
       </c>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A40" s="22"/>
-      <c r="C40" s="13" t="s">
+      <c r="A40" s="17"/>
+      <c r="C40" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="D40" s="13" t="s">
+      <c r="D40" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="E40" s="15" t="s">
+      <c r="E40" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="F40" s="16"/>
-      <c r="G40" s="15" t="s">
+      <c r="F40" s="23"/>
+      <c r="G40" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="H40" s="16"/>
-      <c r="I40" s="19" t="s">
+      <c r="H40" s="23"/>
+      <c r="I40" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="J40" s="20"/>
+      <c r="J40" s="19"/>
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A41" s="22"/>
-      <c r="C41" s="14"/>
-      <c r="D41" s="14"/>
-      <c r="E41" s="17"/>
-      <c r="F41" s="18"/>
-      <c r="G41" s="17"/>
-      <c r="H41" s="18"/>
+      <c r="A41" s="17"/>
+      <c r="C41" s="21"/>
+      <c r="D41" s="21"/>
+      <c r="E41" s="24"/>
+      <c r="F41" s="25"/>
+      <c r="G41" s="24"/>
+      <c r="H41" s="25"/>
       <c r="I41" s="6" t="s">
         <v>36</v>
       </c>
@@ -1490,7 +1491,7 @@
       </c>
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A42" s="22"/>
+      <c r="A42" s="17"/>
       <c r="C42" s="8" t="s">
         <v>54</v>
       </c>
@@ -1510,18 +1511,18 @@
         <v>2</v>
       </c>
       <c r="I42" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="J42" s="8" t="s">
         <v>74</v>
-      </c>
-      <c r="J42" s="8" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="43" spans="1:16" ht="21" x14ac:dyDescent="0.5">
       <c r="B43" s="3"/>
-      <c r="I43" s="25" t="s">
-        <v>73</v>
-      </c>
-      <c r="J43" s="25"/>
+      <c r="I43" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="J43" s="16"/>
     </row>
     <row r="44" spans="1:16" ht="29" x14ac:dyDescent="0.35">
       <c r="A44" s="7" t="s">
@@ -1535,7 +1536,7 @@
         <v>10</v>
       </c>
       <c r="H44" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="45" spans="1:16" ht="21" x14ac:dyDescent="0.5">
@@ -1566,7 +1567,7 @@
     </row>
     <row r="48" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.35">
@@ -1599,30 +1600,30 @@
       <c r="A50" t="s">
         <v>19</v>
       </c>
-      <c r="C50" s="21" t="s">
+      <c r="C50" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="D50" s="21" t="s">
+      <c r="D50" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="E50" s="21" t="s">
+      <c r="E50" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="F50" s="21" t="s">
+      <c r="F50" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="G50" s="21"/>
-      <c r="H50" s="19" t="s">
+      <c r="G50" s="15"/>
+      <c r="H50" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="I50" s="20"/>
+      <c r="I50" s="19"/>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="C51" s="21"/>
-      <c r="D51" s="21"/>
-      <c r="E51" s="21"/>
-      <c r="F51" s="21"/>
-      <c r="G51" s="21"/>
+      <c r="C51" s="15"/>
+      <c r="D51" s="15"/>
+      <c r="E51" s="15"/>
+      <c r="F51" s="15"/>
+      <c r="G51" s="15"/>
       <c r="H51" s="6" t="s">
         <v>36</v>
       </c>
@@ -1662,6 +1663,27 @@
     </row>
   </sheetData>
   <mergeCells count="37">
+    <mergeCell ref="C40:C41"/>
+    <mergeCell ref="D40:D41"/>
+    <mergeCell ref="E40:F41"/>
+    <mergeCell ref="G40:H41"/>
+    <mergeCell ref="I40:J40"/>
+    <mergeCell ref="C50:C51"/>
+    <mergeCell ref="D50:D51"/>
+    <mergeCell ref="E50:E51"/>
+    <mergeCell ref="F50:G51"/>
+    <mergeCell ref="H50:I50"/>
+    <mergeCell ref="A21:A24"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="D22:D23"/>
+    <mergeCell ref="E22:F23"/>
+    <mergeCell ref="G22:H23"/>
+    <mergeCell ref="I22:J22"/>
+    <mergeCell ref="C32:C33"/>
+    <mergeCell ref="D32:D33"/>
+    <mergeCell ref="E32:E33"/>
+    <mergeCell ref="F32:G33"/>
+    <mergeCell ref="H32:I32"/>
     <mergeCell ref="C14:C15"/>
     <mergeCell ref="D14:D15"/>
     <mergeCell ref="I25:J25"/>
@@ -1678,27 +1700,6 @@
     <mergeCell ref="E14:E15"/>
     <mergeCell ref="I7:J7"/>
     <mergeCell ref="A39:A42"/>
-    <mergeCell ref="I22:J22"/>
-    <mergeCell ref="C32:C33"/>
-    <mergeCell ref="D32:D33"/>
-    <mergeCell ref="E32:E33"/>
-    <mergeCell ref="F32:G33"/>
-    <mergeCell ref="H32:I32"/>
-    <mergeCell ref="A21:A24"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="D22:D23"/>
-    <mergeCell ref="E22:F23"/>
-    <mergeCell ref="G22:H23"/>
-    <mergeCell ref="C50:C51"/>
-    <mergeCell ref="D50:D51"/>
-    <mergeCell ref="E50:E51"/>
-    <mergeCell ref="F50:G51"/>
-    <mergeCell ref="H50:I50"/>
-    <mergeCell ref="C40:C41"/>
-    <mergeCell ref="D40:D41"/>
-    <mergeCell ref="E40:F41"/>
-    <mergeCell ref="G40:H41"/>
-    <mergeCell ref="I40:J40"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <hyperlinks>
@@ -1720,11 +1721,11 @@
   <sheetData>
     <row r="1" spans="1:16" ht="21" x14ac:dyDescent="0.5">
       <c r="A1" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="17" t="s">
         <v>8</v>
       </c>
       <c r="B2" t="s">
@@ -1756,34 +1757,34 @@
       </c>
     </row>
     <row r="3" spans="1:16" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="22"/>
-      <c r="C3" s="13" t="s">
+      <c r="A3" s="17"/>
+      <c r="C3" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="E3" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="F3" s="16"/>
-      <c r="G3" s="15" t="s">
+      <c r="F3" s="23"/>
+      <c r="G3" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="H3" s="16"/>
-      <c r="I3" s="19" t="s">
+      <c r="H3" s="23"/>
+      <c r="I3" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="J3" s="20"/>
+      <c r="J3" s="19"/>
     </row>
     <row r="4" spans="1:16" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="22"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="17"/>
-      <c r="F4" s="18"/>
-      <c r="G4" s="17"/>
-      <c r="H4" s="18"/>
+      <c r="A4" s="17"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="25"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="25"/>
       <c r="I4" s="6" t="s">
         <v>36</v>
       </c>
@@ -1792,7 +1793,7 @@
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A5" s="22"/>
+      <c r="A5" s="17"/>
       <c r="C5" s="8" t="s">
         <v>54</v>
       </c>
@@ -1822,14 +1823,14 @@
       <c r="C6" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="26" t="s">
+      <c r="G6" s="28" t="s">
         <v>53</v>
       </c>
-      <c r="H6" s="26"/>
-      <c r="I6" s="26" t="s">
-        <v>77</v>
-      </c>
-      <c r="J6" s="26"/>
+      <c r="H6" s="28"/>
+      <c r="I6" s="28" t="s">
+        <v>76</v>
+      </c>
+      <c r="J6" s="28"/>
     </row>
     <row r="7" spans="1:16" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="7" t="s">
@@ -1844,27 +1845,30 @@
       <c r="C8" t="s">
         <v>14</v>
       </c>
+      <c r="G8" s="1" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A9" s="7"/>
     </row>
-    <row r="10" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="28"/>
-      <c r="B10" s="28"/>
-      <c r="C10" s="28"/>
-      <c r="D10" s="28"/>
-      <c r="E10" s="28"/>
-      <c r="F10" s="28"/>
-      <c r="G10" s="28"/>
-      <c r="H10" s="28"/>
-      <c r="I10" s="28"/>
-      <c r="J10" s="28"/>
-      <c r="K10" s="28"/>
-      <c r="L10" s="28"/>
-      <c r="M10" s="28"/>
-      <c r="N10" s="28"/>
-      <c r="O10" s="28"/>
-      <c r="P10" s="28"/>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A10" s="13"/>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="13"/>
+      <c r="H10" s="13"/>
+      <c r="I10" s="13"/>
+      <c r="J10" s="13"/>
+      <c r="K10" s="13"/>
+      <c r="L10" s="13"/>
+      <c r="M10" s="13"/>
+      <c r="N10" s="13"/>
+      <c r="O10" s="13"/>
+      <c r="P10" s="13"/>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
@@ -1873,7 +1877,7 @@
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.35">
@@ -1909,32 +1913,32 @@
       <c r="A14" t="s">
         <v>19</v>
       </c>
-      <c r="C14" s="13" t="s">
+      <c r="C14" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="D14" s="13" t="s">
+      <c r="D14" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="E14" s="15" t="s">
+      <c r="E14" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="F14" s="16"/>
-      <c r="G14" s="15" t="s">
+      <c r="F14" s="23"/>
+      <c r="G14" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="H14" s="16"/>
-      <c r="I14" s="19" t="s">
+      <c r="H14" s="23"/>
+      <c r="I14" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="J14" s="20"/>
+      <c r="J14" s="19"/>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="17"/>
-      <c r="F15" s="18"/>
-      <c r="G15" s="17"/>
-      <c r="H15" s="18"/>
+      <c r="C15" s="21"/>
+      <c r="D15" s="21"/>
+      <c r="E15" s="24"/>
+      <c r="F15" s="25"/>
+      <c r="G15" s="24"/>
+      <c r="H15" s="25"/>
       <c r="I15" s="6" t="s">
         <v>36</v>
       </c>
@@ -1980,11 +1984,11 @@
     <row r="19" spans="1:16" s="10" customFormat="1" x14ac:dyDescent="0.35"/>
     <row r="20" spans="1:16" ht="21" x14ac:dyDescent="0.5">
       <c r="A20" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A21" s="22" t="s">
+      <c r="A21" s="17" t="s">
         <v>8</v>
       </c>
       <c r="B21" t="s">
@@ -2016,34 +2020,34 @@
       </c>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A22" s="22"/>
-      <c r="C22" s="13" t="s">
+      <c r="A22" s="17"/>
+      <c r="C22" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="D22" s="13" t="s">
+      <c r="D22" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="E22" s="15" t="s">
+      <c r="E22" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="F22" s="16"/>
-      <c r="G22" s="15" t="s">
+      <c r="F22" s="23"/>
+      <c r="G22" s="22" t="s">
         <v>60</v>
       </c>
-      <c r="H22" s="16"/>
-      <c r="I22" s="19" t="s">
+      <c r="H22" s="23"/>
+      <c r="I22" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="J22" s="20"/>
+      <c r="J22" s="19"/>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A23" s="22"/>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="17"/>
-      <c r="F23" s="18"/>
-      <c r="G23" s="17"/>
-      <c r="H23" s="18"/>
+      <c r="A23" s="17"/>
+      <c r="C23" s="21"/>
+      <c r="D23" s="21"/>
+      <c r="E23" s="24"/>
+      <c r="F23" s="25"/>
+      <c r="G23" s="24"/>
+      <c r="H23" s="25"/>
       <c r="I23" s="6" t="s">
         <v>36</v>
       </c>
@@ -2052,7 +2056,7 @@
       </c>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A24" s="22"/>
+      <c r="A24" s="17"/>
       <c r="C24" s="8" t="s">
         <v>2</v>
       </c>
@@ -2072,24 +2076,24 @@
         <v>2</v>
       </c>
       <c r="I24" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="J24" s="8" t="s">
         <v>80</v>
-      </c>
-      <c r="J24" s="8" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="25" spans="1:16" ht="29" x14ac:dyDescent="0.35">
       <c r="C25" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G25" s="26" t="s">
+      <c r="G25" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="H25" s="26"/>
-      <c r="I25" s="26" t="s">
-        <v>79</v>
-      </c>
-      <c r="J25" s="26"/>
+      <c r="H25" s="28"/>
+      <c r="I25" s="28" t="s">
+        <v>78</v>
+      </c>
+      <c r="J25" s="28"/>
     </row>
     <row r="26" spans="1:16" ht="29" x14ac:dyDescent="0.35">
       <c r="A26" s="7" t="s">
@@ -2109,22 +2113,22 @@
       <c r="A28" s="7"/>
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A29" s="28"/>
-      <c r="B29" s="28"/>
-      <c r="C29" s="28"/>
-      <c r="D29" s="28"/>
-      <c r="E29" s="28"/>
-      <c r="F29" s="28"/>
-      <c r="G29" s="28"/>
-      <c r="H29" s="28"/>
-      <c r="I29" s="28"/>
-      <c r="J29" s="28"/>
-      <c r="K29" s="28"/>
-      <c r="L29" s="28"/>
-      <c r="M29" s="28"/>
-      <c r="N29" s="28"/>
-      <c r="O29" s="28"/>
-      <c r="P29" s="28"/>
+      <c r="A29" s="13"/>
+      <c r="B29" s="13"/>
+      <c r="C29" s="13"/>
+      <c r="D29" s="13"/>
+      <c r="E29" s="13"/>
+      <c r="F29" s="13"/>
+      <c r="G29" s="13"/>
+      <c r="H29" s="13"/>
+      <c r="I29" s="13"/>
+      <c r="J29" s="13"/>
+      <c r="K29" s="13"/>
+      <c r="L29" s="13"/>
+      <c r="M29" s="13"/>
+      <c r="N29" s="13"/>
+      <c r="O29" s="13"/>
+      <c r="P29" s="13"/>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A30" s="9" t="s">
@@ -2133,7 +2137,7 @@
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.35">
@@ -2169,32 +2173,32 @@
       <c r="A33" t="s">
         <v>19</v>
       </c>
-      <c r="C33" s="13" t="s">
+      <c r="C33" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="D33" s="13" t="s">
+      <c r="D33" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="E33" s="15" t="s">
+      <c r="E33" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="F33" s="16"/>
-      <c r="G33" s="15" t="s">
+      <c r="F33" s="23"/>
+      <c r="G33" s="22" t="s">
         <v>61</v>
       </c>
-      <c r="H33" s="16"/>
-      <c r="I33" s="19" t="s">
+      <c r="H33" s="23"/>
+      <c r="I33" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="J33" s="20"/>
+      <c r="J33" s="19"/>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="C34" s="14"/>
-      <c r="D34" s="14"/>
-      <c r="E34" s="17"/>
-      <c r="F34" s="18"/>
-      <c r="G34" s="17"/>
-      <c r="H34" s="18"/>
+      <c r="C34" s="21"/>
+      <c r="D34" s="21"/>
+      <c r="E34" s="24"/>
+      <c r="F34" s="25"/>
+      <c r="G34" s="24"/>
+      <c r="H34" s="25"/>
       <c r="I34" s="6" t="s">
         <v>36</v>
       </c>
@@ -2238,14 +2242,15 @@
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="I22:J22"/>
-    <mergeCell ref="G25:H25"/>
-    <mergeCell ref="I25:J25"/>
-    <mergeCell ref="C33:C34"/>
-    <mergeCell ref="D33:D34"/>
-    <mergeCell ref="E33:F34"/>
-    <mergeCell ref="G33:H34"/>
-    <mergeCell ref="I33:J33"/>
+    <mergeCell ref="I14:J14"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E3:F4"/>
+    <mergeCell ref="G3:H4"/>
     <mergeCell ref="C14:C15"/>
     <mergeCell ref="D14:D15"/>
     <mergeCell ref="E14:F15"/>
@@ -2255,16 +2260,18 @@
     <mergeCell ref="D22:D23"/>
     <mergeCell ref="E22:F23"/>
     <mergeCell ref="G22:H23"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="E3:F4"/>
-    <mergeCell ref="G3:H4"/>
-    <mergeCell ref="I14:J14"/>
+    <mergeCell ref="I22:J22"/>
+    <mergeCell ref="G25:H25"/>
+    <mergeCell ref="I25:J25"/>
+    <mergeCell ref="C33:C34"/>
+    <mergeCell ref="D33:D34"/>
+    <mergeCell ref="E33:F34"/>
+    <mergeCell ref="G33:H34"/>
+    <mergeCell ref="I33:J33"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="G8" r:id="rId1" xr:uid="{12BD2609-7915-4B96-828E-BBF6EE96881F}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2284,7 +2291,7 @@
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="17" t="s">
         <v>8</v>
       </c>
       <c r="B2" t="s">
@@ -2316,34 +2323,34 @@
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A3" s="22"/>
-      <c r="C3" s="13" t="s">
+      <c r="A3" s="17"/>
+      <c r="C3" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="E3" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="F3" s="16"/>
-      <c r="G3" s="15" t="s">
+      <c r="F3" s="23"/>
+      <c r="G3" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="H3" s="16"/>
-      <c r="I3" s="19" t="s">
+      <c r="H3" s="23"/>
+      <c r="I3" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="J3" s="20"/>
+      <c r="J3" s="19"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A4" s="22"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="17"/>
-      <c r="F4" s="18"/>
-      <c r="G4" s="17"/>
-      <c r="H4" s="18"/>
+      <c r="A4" s="17"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="25"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="25"/>
       <c r="I4" s="6" t="s">
         <v>36</v>
       </c>
@@ -2352,7 +2359,7 @@
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A5" s="22"/>
+      <c r="A5" s="17"/>
       <c r="C5" s="8" t="s">
         <v>25</v>
       </c>
@@ -2382,10 +2389,10 @@
       <c r="C6" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="26"/>
-      <c r="H6" s="26"/>
-      <c r="I6" s="26"/>
-      <c r="J6" s="26"/>
+      <c r="G6" s="28"/>
+      <c r="H6" s="28"/>
+      <c r="I6" s="28"/>
+      <c r="J6" s="28"/>
     </row>
     <row r="7" spans="1:16" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="7" t="s">
@@ -2396,23 +2403,23 @@
         <v>FF 03 07 D0 00 01 91 59</v>
       </c>
     </row>
-    <row r="9" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="29"/>
-      <c r="B9" s="29"/>
-      <c r="C9" s="29"/>
-      <c r="D9" s="29"/>
-      <c r="E9" s="29"/>
-      <c r="F9" s="29"/>
-      <c r="G9" s="29"/>
-      <c r="H9" s="29"/>
-      <c r="I9" s="29"/>
-      <c r="J9" s="29"/>
-      <c r="K9" s="29"/>
-      <c r="L9" s="29"/>
-      <c r="M9" s="29"/>
-      <c r="N9" s="29"/>
-      <c r="O9" s="29"/>
-      <c r="P9" s="29"/>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A9" s="14"/>
+      <c r="B9" s="14"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="14"/>
+      <c r="I9" s="14"/>
+      <c r="J9" s="14"/>
+      <c r="K9" s="14"/>
+      <c r="L9" s="14"/>
+      <c r="M9" s="14"/>
+      <c r="N9" s="14"/>
+      <c r="O9" s="14"/>
+      <c r="P9" s="14"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A10" s="9" t="s">
@@ -2421,7 +2428,7 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>62</v>
+        <v>90</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.35">
@@ -2454,30 +2461,30 @@
       <c r="A13" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="13" t="s">
+      <c r="C13" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="D13" s="13" t="s">
+      <c r="D13" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="E13" s="13" t="s">
+      <c r="E13" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="F13" s="15" t="s">
+      <c r="F13" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="G13" s="16"/>
-      <c r="H13" s="19" t="s">
+      <c r="G13" s="23"/>
+      <c r="H13" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="I13" s="20"/>
+      <c r="I13" s="19"/>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="17"/>
-      <c r="G14" s="18"/>
+      <c r="C14" s="21"/>
+      <c r="D14" s="21"/>
+      <c r="E14" s="21"/>
+      <c r="F14" s="24"/>
+      <c r="G14" s="25"/>
       <c r="H14" s="6" t="s">
         <v>36</v>
       </c>
@@ -2488,7 +2495,7 @@
     <row r="15" spans="1:16" x14ac:dyDescent="0.35">
       <c r="C15" s="5" t="str">
         <f>"0x"&amp;MID(SUBSTITUTE(SUBSTITUTE($A$11,"{",""),"}",""),(COLUMN(A11)-1)*2+1,2)</f>
-        <v>0x01</v>
+        <v>0x07</v>
       </c>
       <c r="D15" s="5" t="str">
         <f t="shared" ref="D15:I15" si="0">"0x"&amp;MID(SUBSTITUTE(SUBSTITUTE($A$11,"{",""),"}",""),(COLUMN(B11)-1)*2+1,2)</f>
@@ -2504,40 +2511,31 @@
       </c>
       <c r="G15" s="5" t="str">
         <f t="shared" si="0"/>
-        <v>0x01</v>
+        <v>0x07</v>
       </c>
       <c r="H15" s="5" t="str">
         <f t="shared" si="0"/>
-        <v>0x79</v>
+        <v>0x71</v>
       </c>
       <c r="I15" s="5" t="str">
         <f t="shared" si="0"/>
-        <v>0x84</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="C16" s="30"/>
-      <c r="D16" s="30"/>
-      <c r="E16" s="30"/>
-      <c r="F16" s="30"/>
-      <c r="G16" s="30"/>
-      <c r="H16" s="30"/>
-      <c r="I16" s="30"/>
+        <v>0x86</v>
+      </c>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.35">
       <c r="C17" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="19" spans="1:16" s="10" customFormat="1" x14ac:dyDescent="0.35"/>
     <row r="20" spans="1:16" s="10" customFormat="1" x14ac:dyDescent="0.35"/>
     <row r="22" spans="1:16" ht="21" x14ac:dyDescent="0.5">
       <c r="A22" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A23" s="22" t="s">
+      <c r="A23" s="17" t="s">
         <v>8</v>
       </c>
       <c r="B23" t="s">
@@ -2568,38 +2566,38 @@
         <v>7</v>
       </c>
       <c r="L23" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A24" s="22"/>
-      <c r="C24" s="13" t="s">
+      <c r="A24" s="17"/>
+      <c r="C24" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="D24" s="13" t="s">
+      <c r="D24" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="E24" s="15" t="s">
+      <c r="E24" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="F24" s="16"/>
-      <c r="G24" s="15" t="s">
+      <c r="F24" s="23"/>
+      <c r="G24" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="H24" s="16"/>
-      <c r="I24" s="19" t="s">
+      <c r="H24" s="23"/>
+      <c r="I24" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="J24" s="20"/>
+      <c r="J24" s="19"/>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A25" s="22"/>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="17"/>
-      <c r="F25" s="18"/>
-      <c r="G25" s="17"/>
-      <c r="H25" s="18"/>
+      <c r="A25" s="17"/>
+      <c r="C25" s="21"/>
+      <c r="D25" s="21"/>
+      <c r="E25" s="24"/>
+      <c r="F25" s="25"/>
+      <c r="G25" s="24"/>
+      <c r="H25" s="25"/>
       <c r="I25" s="6" t="s">
         <v>36</v>
       </c>
@@ -2608,7 +2606,7 @@
       </c>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A26" s="22"/>
+      <c r="A26" s="17"/>
       <c r="C26" s="8" t="s">
         <v>25</v>
       </c>
@@ -2638,12 +2636,12 @@
       <c r="C27" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G27" s="26"/>
-      <c r="H27" s="26"/>
-      <c r="I27" s="26" t="s">
+      <c r="G27" s="28"/>
+      <c r="H27" s="28"/>
+      <c r="I27" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="J27" s="26"/>
+      <c r="J27" s="28"/>
     </row>
     <row r="28" spans="1:16" ht="29" x14ac:dyDescent="0.35">
       <c r="A28" s="7" t="s">
@@ -2655,22 +2653,22 @@
       </c>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A30" s="29"/>
-      <c r="B30" s="29"/>
-      <c r="C30" s="29"/>
-      <c r="D30" s="29"/>
-      <c r="E30" s="29"/>
-      <c r="F30" s="29"/>
-      <c r="G30" s="29"/>
-      <c r="H30" s="29"/>
-      <c r="I30" s="29"/>
-      <c r="J30" s="29"/>
-      <c r="K30" s="29"/>
-      <c r="L30" s="29"/>
-      <c r="M30" s="29"/>
-      <c r="N30" s="29"/>
-      <c r="O30" s="29"/>
-      <c r="P30" s="29"/>
+      <c r="A30" s="14"/>
+      <c r="B30" s="14"/>
+      <c r="C30" s="14"/>
+      <c r="D30" s="14"/>
+      <c r="E30" s="14"/>
+      <c r="F30" s="14"/>
+      <c r="G30" s="14"/>
+      <c r="H30" s="14"/>
+      <c r="I30" s="14"/>
+      <c r="J30" s="14"/>
+      <c r="K30" s="14"/>
+      <c r="L30" s="14"/>
+      <c r="M30" s="14"/>
+      <c r="N30" s="14"/>
+      <c r="O30" s="14"/>
+      <c r="P30" s="14"/>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A31" s="9" t="s">
@@ -2679,7 +2677,7 @@
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.35">
@@ -2712,30 +2710,30 @@
       <c r="A34" t="s">
         <v>19</v>
       </c>
-      <c r="C34" s="13" t="s">
+      <c r="C34" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="D34" s="13" t="s">
+      <c r="D34" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="E34" s="13" t="s">
+      <c r="E34" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="F34" s="15" t="s">
+      <c r="F34" s="22" t="s">
         <v>60</v>
       </c>
-      <c r="G34" s="16"/>
-      <c r="H34" s="19" t="s">
+      <c r="G34" s="23"/>
+      <c r="H34" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="I34" s="20"/>
+      <c r="I34" s="19"/>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="C35" s="14"/>
-      <c r="D35" s="14"/>
-      <c r="E35" s="14"/>
-      <c r="F35" s="17"/>
-      <c r="G35" s="18"/>
+      <c r="C35" s="21"/>
+      <c r="D35" s="21"/>
+      <c r="E35" s="21"/>
+      <c r="F35" s="24"/>
+      <c r="G35" s="25"/>
       <c r="H35" s="6" t="s">
         <v>36</v>
       </c>
@@ -2780,19 +2778,6 @@
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="G27:H27"/>
-    <mergeCell ref="I27:J27"/>
-    <mergeCell ref="C34:C35"/>
-    <mergeCell ref="D34:D35"/>
-    <mergeCell ref="E34:E35"/>
-    <mergeCell ref="F34:G35"/>
-    <mergeCell ref="H34:I34"/>
-    <mergeCell ref="F13:G14"/>
-    <mergeCell ref="A23:A26"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="E24:F25"/>
-    <mergeCell ref="G24:H25"/>
     <mergeCell ref="I24:J24"/>
     <mergeCell ref="H13:I13"/>
     <mergeCell ref="A2:A5"/>
@@ -2806,6 +2791,19 @@
     <mergeCell ref="C13:C14"/>
     <mergeCell ref="D13:D14"/>
     <mergeCell ref="E13:E14"/>
+    <mergeCell ref="F13:G14"/>
+    <mergeCell ref="A23:A26"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="E24:F25"/>
+    <mergeCell ref="G24:H25"/>
+    <mergeCell ref="G27:H27"/>
+    <mergeCell ref="I27:J27"/>
+    <mergeCell ref="C34:C35"/>
+    <mergeCell ref="D34:D35"/>
+    <mergeCell ref="E34:E35"/>
+    <mergeCell ref="F34:G35"/>
+    <mergeCell ref="H34:I34"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2857,14 +2855,14 @@
       <c r="D3" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="19" t="s">
+      <c r="E3" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="F3" s="20"/>
-      <c r="G3" s="19" t="s">
+      <c r="F3" s="19"/>
+      <c r="G3" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="H3" s="20"/>
+      <c r="H3" s="19"/>
       <c r="I3" s="6" t="s">
         <v>23</v>
       </c>

</xml_diff>